<commit_message>
Optimize Excel parsing pipeline using Promise.all batching and defer dashboard refresh
</commit_message>
<xml_diff>
--- a/Sample_Clients.xlsx
+++ b/Sample_Clients.xlsx
@@ -1,44 +1,176 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr codeName="ThisWorkbook"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Diamond\diamondpr\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3807D76-96AC-4E48-83D9-5F3229695855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="11808" yWindow="2460" windowWidth="11172" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="Clients" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="45">
+  <si>
+    <t>ClientCode</t>
+  </si>
+  <si>
+    <t>CompanyName</t>
+  </si>
+  <si>
+    <t>ContactNo</t>
+  </si>
+  <si>
+    <t>ContactName</t>
+  </si>
+  <si>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>GSTNumber</t>
+  </si>
+  <si>
+    <t>Industry</t>
+  </si>
+  <si>
+    <t>Remarks</t>
+  </si>
+  <si>
+    <t>Tech Innovators Inc</t>
+  </si>
+  <si>
+    <t>+91 9876543210</t>
+  </si>
+  <si>
+    <t>Rahul Sharma</t>
+  </si>
+  <si>
+    <t>rahul@techinnovators.com</t>
+  </si>
+  <si>
+    <t>123 Tech Park, Bangalore</t>
+  </si>
+  <si>
+    <t>29ABCDE1234F1Z5</t>
+  </si>
+  <si>
+    <t>IT / Software</t>
+  </si>
+  <si>
+    <t>Priority client, needs weekly follow-ups</t>
+  </si>
+  <si>
+    <t>Global Logistics Solutions</t>
+  </si>
+  <si>
+    <t>+44 7911123456</t>
+  </si>
+  <si>
+    <t>Sarah Jenkins</t>
+  </si>
+  <si>
+    <t>s.jenkins@globallogistics.co.uk</t>
+  </si>
+  <si>
+    <t>45 Freight Way, London</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Logistics</t>
+  </si>
+  <si>
+    <t>Looking for annual contract</t>
+  </si>
+  <si>
+    <t>Green Energy Corp</t>
+  </si>
+  <si>
+    <t>+1 5550198765</t>
+  </si>
+  <si>
+    <t>Michael Green</t>
+  </si>
+  <si>
+    <t>mgreen@greenenergy.com</t>
+  </si>
+  <si>
+    <t>789 Eco Ave, California</t>
+  </si>
+  <si>
+    <t>12XYZDE5678G2Z1</t>
+  </si>
+  <si>
+    <t>Renewable Energy</t>
+  </si>
+  <si>
+    <t>Interested in bulk orders</t>
+  </si>
+  <si>
+    <t>Apex Manufacturing</t>
+  </si>
+  <si>
+    <t>+91 8765432109</t>
+  </si>
+  <si>
+    <t>Anita Desai</t>
+  </si>
+  <si>
+    <t>anita@apexmanufacturing.in</t>
+  </si>
+  <si>
+    <t>Plot 42, Industrial Area, Pune</t>
+  </si>
+  <si>
+    <t>27PQRST4321M1Z2</t>
+  </si>
+  <si>
+    <t>Manufacturing</t>
+  </si>
+  <si>
+    <t>Requires custom quotations</t>
+  </si>
+  <si>
+    <t>BULK-008</t>
+  </si>
+  <si>
+    <t>BULK-009</t>
+  </si>
+  <si>
+    <t>BULK-010</t>
+  </si>
+  <si>
+    <t>BULK-011</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -65,13 +197,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,157 +536,160 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I5"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>ClientCode</v>
-      </c>
-      <c r="B1" t="str">
-        <v>CompanyName</v>
-      </c>
-      <c r="C1" t="str">
-        <v>ContactNo</v>
-      </c>
-      <c r="D1" t="str">
-        <v>ContactName</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Email</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Address</v>
-      </c>
-      <c r="G1" t="str">
-        <v>GSTNumber</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Industry</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Remarks</v>
+    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>BULK-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Tech Innovators Inc</v>
-      </c>
-      <c r="C2" t="str">
-        <v>+91 9876543210</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Rahul Sharma</v>
-      </c>
-      <c r="E2" t="str">
-        <v>rahul@techinnovators.com</v>
-      </c>
-      <c r="F2" t="str">
-        <v>123 Tech Park, Bangalore</v>
-      </c>
-      <c r="G2" t="str">
-        <v>29ABCDE1234F1Z5</v>
-      </c>
-      <c r="H2" t="str">
-        <v>IT / Software</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Priority client, needs weekly follow-ups</v>
+    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G2" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" t="s">
+        <v>16</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>BULK-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Global Logistics Solutions</v>
-      </c>
-      <c r="C3" t="str">
-        <v>+44 7911123456</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Sarah Jenkins</v>
-      </c>
-      <c r="E3" t="str">
-        <v>s.jenkins@globallogistics.co.uk</v>
-      </c>
-      <c r="F3" t="str">
-        <v>45 Freight Way, London</v>
-      </c>
-      <c r="G3" t="str">
-        <v/>
-      </c>
-      <c r="H3" t="str">
-        <v>Logistics</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Looking for annual contract</v>
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+      <c r="E3" t="s">
+        <v>20</v>
+      </c>
+      <c r="F3" t="s">
+        <v>21</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
+        <v>23</v>
+      </c>
+      <c r="I3" t="s">
+        <v>24</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>BULK-003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Green Energy Corp</v>
-      </c>
-      <c r="C4" t="str">
-        <v>+1 5550198765</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Michael Green</v>
-      </c>
-      <c r="E4" t="str">
-        <v>mgreen@greenenergy.com</v>
-      </c>
-      <c r="F4" t="str">
-        <v>789 Eco Ave, California</v>
-      </c>
-      <c r="G4" t="str">
-        <v>12XYZDE5678G2Z1</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Renewable Energy</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Interested in bulk orders</v>
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G4" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" t="s">
+        <v>31</v>
+      </c>
+      <c r="I4" t="s">
+        <v>32</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>BULK-004</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Apex Manufacturing</v>
-      </c>
-      <c r="C5" t="str">
-        <v>+91 8765432109</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Anita Desai</v>
-      </c>
-      <c r="E5" t="str">
-        <v>anita@apexmanufacturing.in</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Plot 42, Industrial Area, Pune</v>
-      </c>
-      <c r="G5" t="str">
-        <v>27PQRST4321M1Z2</v>
-      </c>
-      <c r="H5" t="str">
-        <v>Manufacturing</v>
-      </c>
-      <c r="I5" t="str">
-        <v>Requires custom quotations</v>
+    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s">
+        <v>34</v>
+      </c>
+      <c r="D5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E5" t="s">
+        <v>36</v>
+      </c>
+      <c r="F5" t="s">
+        <v>37</v>
+      </c>
+      <c r="G5" t="s">
+        <v>38</v>
+      </c>
+      <c r="H5" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" t="s">
+        <v>40</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I5"/>
+    <ignoredError sqref="A1:I1 B4:I5 B2:I2 B3:I3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix DatePickerInput imports and uploadPrimaryContactProfileImage type in ERPContext
</commit_message>
<xml_diff>
--- a/Sample_Clients.xlsx
+++ b/Sample_Clients.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hp\Downloads\Diamond\diamondpr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3807D76-96AC-4E48-83D9-5F3229695855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D6070F4-CE19-4708-BFC1-4EB2E5993A67}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="11808" yWindow="2460" windowWidth="11172" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -145,16 +145,16 @@
     <t>Requires custom quotations</t>
   </si>
   <si>
-    <t>BULK-008</t>
-  </si>
-  <si>
-    <t>BULK-009</t>
-  </si>
-  <si>
-    <t>BULK-010</t>
-  </si>
-  <si>
-    <t>BULK-011</t>
+    <t>BULK-020</t>
+  </si>
+  <si>
+    <t>BULK-021</t>
+  </si>
+  <si>
+    <t>BULK-022</t>
+  </si>
+  <si>
+    <t>BULK-023</t>
   </si>
 </sst>
 </file>
@@ -538,9 +538,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I5"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -569,7 +569,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -598,7 +598,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -627,7 +627,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>43</v>
       </c>
@@ -656,7 +656,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>44</v>
       </c>

</xml_diff>